<commit_message>
chore(data): pipeline OK [price-only] 2026-09-11 13:09
</commit_message>
<xml_diff>
--- a/data/0_raw/exchange_rate_data.xlsx
+++ b/data/0_raw/exchange_rate_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1650"/>
+  <dimension ref="A1:B1651"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16930,6 +16930,16 @@
         <v>1338.9</v>
       </c>
     </row>
+    <row r="1651">
+      <c r="A1651" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B1651" t="n">
+        <v>1344.6</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(data): pipeline OK [full] 2026-09-15 08:06
</commit_message>
<xml_diff>
--- a/data/0_raw/exchange_rate_data.xlsx
+++ b/data/0_raw/exchange_rate_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1651"/>
+  <dimension ref="A1:B1652"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16940,6 +16940,16 @@
         <v>1344.6</v>
       </c>
     </row>
+    <row r="1652">
+      <c r="A1652" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B1652" t="n">
+        <v>1348.5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(data): pipeline OK [price-only] 2026-09-17 09:13
</commit_message>
<xml_diff>
--- a/data/0_raw/exchange_rate_data.xlsx
+++ b/data/0_raw/exchange_rate_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1652"/>
+  <dimension ref="A1:B1655"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16950,6 +16950,36 @@
         <v>1348.5</v>
       </c>
     </row>
+    <row r="1653">
+      <c r="A1653" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1653" t="n">
+        <v>1363.7</v>
+      </c>
+    </row>
+    <row r="1654">
+      <c r="A1654" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1654" t="n">
+        <v>1377.5</v>
+      </c>
+    </row>
+    <row r="1655">
+      <c r="A1655" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1655" t="n">
+        <v>1375.2</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(data): pipeline OK [price-only] 2026-09-18 08:04
</commit_message>
<xml_diff>
--- a/data/0_raw/exchange_rate_data.xlsx
+++ b/data/0_raw/exchange_rate_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1655"/>
+  <dimension ref="A1:B1656"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16980,6 +16980,18 @@
         <v>1375.2</v>
       </c>
     </row>
+    <row r="1656">
+      <c r="A1656" t="inlineStr">
+        <is>
+          <t>이 페이지는 더 이상 제공되지 않습니다- Npay 증권 바로가기</t>
+        </is>
+      </c>
+      <c r="B1656" t="inlineStr">
+        <is>
+          <t>이 페이지는 더 이상 제공되지 않습니다. Npay 증권 바로가기</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(data): pipeline OK [price-only] 2026-10-13 17:02
</commit_message>
<xml_diff>
--- a/data/0_raw/exchange_rate_data.xlsx
+++ b/data/0_raw/exchange_rate_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1915"/>
+  <dimension ref="A1:B1916"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19580,6 +19580,16 @@
         <v>1338</v>
       </c>
     </row>
+    <row r="1916">
+      <c r="A1916" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B1916" t="n">
+        <v>1335.8</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(data): pipeline OK [price-only] 2026-10-15 08:04
</commit_message>
<xml_diff>
--- a/data/0_raw/exchange_rate_data.xlsx
+++ b/data/0_raw/exchange_rate_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1916"/>
+  <dimension ref="A1:B1917"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19590,6 +19590,16 @@
         <v>1335.8</v>
       </c>
     </row>
+    <row r="1917">
+      <c r="A1917" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B1917" t="n">
+        <v>1340.5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(data): pipeline OK [price-only] 2026-10-16 08:03
</commit_message>
<xml_diff>
--- a/data/0_raw/exchange_rate_data.xlsx
+++ b/data/0_raw/exchange_rate_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1917"/>
+  <dimension ref="A1:B1918"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19600,6 +19600,16 @@
         <v>1340.5</v>
       </c>
     </row>
+    <row r="1918">
+      <c r="A1918" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B1918" t="n">
+        <v>1338.6</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(data): pipeline OK [price-only] 2026-10-19 08:03
</commit_message>
<xml_diff>
--- a/data/0_raw/exchange_rate_data.xlsx
+++ b/data/0_raw/exchange_rate_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1918"/>
+  <dimension ref="A1:B1919"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19610,6 +19610,16 @@
         <v>1338.6</v>
       </c>
     </row>
+    <row r="1919">
+      <c r="A1919" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B1919" t="n">
+        <v>1348.5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(data): pipeline OK [full] 2026-10-20 08:18
</commit_message>
<xml_diff>
--- a/data/0_raw/exchange_rate_data.xlsx
+++ b/data/0_raw/exchange_rate_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1919"/>
+  <dimension ref="A1:B1920"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19620,6 +19620,16 @@
         <v>1348.5</v>
       </c>
     </row>
+    <row r="1920">
+      <c r="A1920" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B1920" t="n">
+        <v>1342.4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(data): pipeline OK [price-only] 2026-10-22 08:07
</commit_message>
<xml_diff>
--- a/data/0_raw/exchange_rate_data.xlsx
+++ b/data/0_raw/exchange_rate_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1920"/>
+  <dimension ref="A1:B1922"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19630,6 +19630,26 @@
         <v>1342.4</v>
       </c>
     </row>
+    <row r="1921">
+      <c r="A1921" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B1921" t="n">
+        <v>1332.1</v>
+      </c>
+    </row>
+    <row r="1922">
+      <c r="A1922" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B1922" t="n">
+        <v>1328</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(data): pipeline OK [price-only] 2026-10-23 08:12
</commit_message>
<xml_diff>
--- a/data/0_raw/exchange_rate_data.xlsx
+++ b/data/0_raw/exchange_rate_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1922"/>
+  <dimension ref="A1:B1923"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19650,6 +19650,16 @@
         <v>1328</v>
       </c>
     </row>
+    <row r="1923">
+      <c r="A1923" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B1923" t="n">
+        <v>1325.5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(data): pipeline OK [price-only] 2026-10-27 07:57
</commit_message>
<xml_diff>
--- a/data/0_raw/exchange_rate_data.xlsx
+++ b/data/0_raw/exchange_rate_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1923"/>
+  <dimension ref="A1:B1925"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19660,6 +19660,26 @@
         <v>1325.5</v>
       </c>
     </row>
+    <row r="1924">
+      <c r="A1924" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B1924" t="n">
+        <v>1324.6</v>
+      </c>
+    </row>
+    <row r="1925">
+      <c r="A1925" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B1925" t="n">
+        <v>1324.3</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(data): pipeline OK [full] 2026-10-28 08:18
</commit_message>
<xml_diff>
--- a/data/0_raw/exchange_rate_data.xlsx
+++ b/data/0_raw/exchange_rate_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1925"/>
+  <dimension ref="A1:B1926"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19680,6 +19680,16 @@
         <v>1324.3</v>
       </c>
     </row>
+    <row r="1926">
+      <c r="A1926" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B1926" t="n">
+        <v>1322.6</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(data): pipeline OK [full] 2026-10-29 08:14
</commit_message>
<xml_diff>
--- a/data/0_raw/exchange_rate_data.xlsx
+++ b/data/0_raw/exchange_rate_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1926"/>
+  <dimension ref="A1:B1927"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19690,6 +19690,16 @@
         <v>1322.6</v>
       </c>
     </row>
+    <row r="1927">
+      <c r="A1927" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B1927" t="n">
+        <v>1324.3</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(data): pipeline OK [full] 2026-10-30 08:25
</commit_message>
<xml_diff>
--- a/data/0_raw/exchange_rate_data.xlsx
+++ b/data/0_raw/exchange_rate_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1927"/>
+  <dimension ref="A1:B1928"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19700,6 +19700,16 @@
         <v>1324.3</v>
       </c>
     </row>
+    <row r="1928">
+      <c r="A1928" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="B1928" t="n">
+        <v>1336.3</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>